<commit_message>
Improve stability by adding unique keys to lists and elements
Add stable `key` props to repeated elements and lists within the Estimating Module page to resolve React warnings and ensure proper rendering.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 122ba5df-9fd5-4238-810a-9bf103a8fecb
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/9ejOnDb
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-08.xlsx
+++ b/backups/proposal-log-2026-04-08.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="115">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -284,6 +284,9 @@
   </si>
   <si>
     <t>Vahid Balali</t>
+  </si>
+  <si>
+    <t>80033</t>
   </si>
   <si>
     <t>2026-06-01</t>
@@ -1277,48 +1280,48 @@
         <v>90</v>
       </c>
       <c r="I12" t="s">
-        <v>56</v>
+        <v>91</v>
       </c>
       <c r="J12" t="s">
         <v>57</v>
       </c>
       <c r="K12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="M12" t="s">
         <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G13" t="s">
         <v>83</v>
       </c>
       <c r="H13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I13" t="s">
         <v>56</v>
@@ -1336,33 +1339,33 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E14" t="s">
         <v>54</v>
       </c>
       <c r="F14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G14" t="s">
         <v>17</v>
       </c>
       <c r="H14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I14" t="s">
         <v>17</v>
@@ -1380,18 +1383,18 @@
         <v>17</v>
       </c>
       <c r="N14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D15" t="s">
         <v>77</v>
@@ -1406,7 +1409,7 @@
         <v>17</v>
       </c>
       <c r="H15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I15" t="s">
         <v>56</v>
@@ -1424,18 +1427,18 @@
         <v>17</v>
       </c>
       <c r="N15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D16" t="s">
         <v>77</v>
@@ -1450,7 +1453,7 @@
         <v>17</v>
       </c>
       <c r="H16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I16" t="s">
         <v>17</v>
@@ -1468,7 +1471,7 @@
         <v>17</v>
       </c>
       <c r="N16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update user permissions and role labels for improved access management
Introduces role label changes for "Standard User" to "Estimator" and "Full Access" to "Admin". Implements functionality to grant and revoke individual user features temporarily via new mutations and updates the UI to reflect these changes. The `AdminUserPermissionsPage` now uses `useMemo` for user deduplication and `useEffect` to manage initial user feature state, also fixing a rendering loop bug by memoizing a dependency. Schema changes in `shared/schema.ts` define the `ROLE_LABELS` constant.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 69b50297-64cc-4fc0-a364-4ee7ddfbc7e9
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/9ejOnDb
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-08.xlsx
+++ b/backups/proposal-log-2026-04-08.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="122">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -178,6 +178,9 @@
     <t>2026-04-03</t>
   </si>
   <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
     <t>Nick Jennings</t>
   </si>
   <si>
@@ -250,9 +253,6 @@
     <t>2026-03-31</t>
   </si>
   <si>
-    <t>2026-04-13</t>
-  </si>
-  <si>
     <t>Jake Marrujo</t>
   </si>
   <si>
@@ -274,7 +274,7 @@
     <t>Illumina Project SOL</t>
   </si>
   <si>
-    <t>SAN</t>
+    <t>SAN - SD</t>
   </si>
   <si>
     <t>2026-04-21</t>
@@ -286,7 +286,7 @@
     <t>Vahid Balali</t>
   </si>
   <si>
-    <t>80033</t>
+    <t>148686</t>
   </si>
   <si>
     <t>2026-06-01</t>
@@ -356,6 +356,27 @@
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69d3de61132a4642c558b4df</t>
+  </si>
+  <si>
+    <t>26-0219</t>
+  </si>
+  <si>
+    <t>Station 33 Bldg 4 Food Hall SD Budget</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>Jonathan Enriquez</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d403f406964200385d4f8c</t>
+  </si>
+  <si>
+    <t>26-0218</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d3dce067942824a3512727</t>
   </si>
 </sst>
 </file>
@@ -754,7 +775,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1007,19 +1028,19 @@
         <v>54</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="G6" t="s">
         <v>17</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K6" t="s">
         <v>17</v>
@@ -1031,18 +1052,18 @@
         <v>17</v>
       </c>
       <c r="N6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
         <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
         <v>45</v>
@@ -1057,13 +1078,13 @@
         <v>17</v>
       </c>
       <c r="H7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I7" t="s">
         <v>17</v>
       </c>
       <c r="J7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K7" t="s">
         <v>17</v>
@@ -1075,18 +1096,18 @@
         <v>17</v>
       </c>
       <c r="N7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D8" t="s">
         <v>17</v>
@@ -1095,19 +1116,19 @@
         <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G8" t="s">
         <v>17</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I8" t="s">
         <v>17</v>
       </c>
       <c r="J8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K8" t="s">
         <v>17</v>
@@ -1119,15 +1140,15 @@
         <v>17</v>
       </c>
       <c r="N8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C9" t="s">
         <v>53</v>
@@ -1139,19 +1160,19 @@
         <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G9" t="s">
         <v>17</v>
       </c>
       <c r="H9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
         <v>17</v>
       </c>
       <c r="J9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K9" t="s">
         <v>17</v>
@@ -1163,27 +1184,27 @@
         <v>17</v>
       </c>
       <c r="N9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F10" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="G10" t="s">
         <v>17</v>
@@ -1195,7 +1216,7 @@
         <v>17</v>
       </c>
       <c r="J10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K10" t="s">
         <v>17</v>
@@ -1239,7 +1260,7 @@
         <v>84</v>
       </c>
       <c r="J11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K11" t="s">
         <v>17</v>
@@ -1265,7 +1286,7 @@
         <v>87</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E12" t="s">
         <v>18</v>
@@ -1283,7 +1304,7 @@
         <v>91</v>
       </c>
       <c r="J12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K12" t="s">
         <v>92</v>
@@ -1324,10 +1345,10 @@
         <v>100</v>
       </c>
       <c r="I13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K13" t="s">
         <v>17</v>
@@ -1371,7 +1392,7 @@
         <v>17</v>
       </c>
       <c r="J14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K14" t="s">
         <v>17</v>
@@ -1397,7 +1418,7 @@
         <v>110</v>
       </c>
       <c r="D15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E15" t="s">
         <v>37</v>
@@ -1412,10 +1433,10 @@
         <v>111</v>
       </c>
       <c r="I15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K15" t="s">
         <v>17</v>
@@ -1441,7 +1462,7 @@
         <v>110</v>
       </c>
       <c r="D16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
@@ -1459,7 +1480,7 @@
         <v>17</v>
       </c>
       <c r="J16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K16" t="s">
         <v>17</v>
@@ -1474,8 +1495,96 @@
         <v>114</v>
       </c>
     </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>115</v>
+      </c>
+      <c r="B17" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" t="s">
+        <v>78</v>
+      </c>
+      <c r="E17" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" t="s">
+        <v>117</v>
+      </c>
+      <c r="G17" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" t="s">
+        <v>118</v>
+      </c>
+      <c r="I17" t="s">
+        <v>17</v>
+      </c>
+      <c r="J17" t="s">
+        <v>58</v>
+      </c>
+      <c r="K17" t="s">
+        <v>17</v>
+      </c>
+      <c r="L17" t="s">
+        <v>17</v>
+      </c>
+      <c r="M17" t="s">
+        <v>17</v>
+      </c>
+      <c r="N17" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" t="s">
+        <v>88</v>
+      </c>
+      <c r="G18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" t="s">
+        <v>111</v>
+      </c>
+      <c r="I18" t="s">
+        <v>17</v>
+      </c>
+      <c r="J18" t="s">
+        <v>58</v>
+      </c>
+      <c r="K18" t="s">
+        <v>17</v>
+      </c>
+      <c r="L18" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" t="s">
+        <v>17</v>
+      </c>
+      <c r="N18" t="s">
+        <v>121</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N16"/>
+  <autoFilter ref="A1:N18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>